<commit_message>
Modif du tableau de synthèse
</commit_message>
<xml_diff>
--- a/public/Tableau de synthese.xlsx
+++ b/public/Tableau de synthese.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9BE7A464-BBA2-4798-AEF1-145E54BA1713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1E34428-B898-4FA9-987F-F34C0426BCBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$29</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="58">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -48,9 +48,6 @@
   </si>
   <si>
     <t xml:space="preserve">Tableau de synthèse des réalisations professionnelles </t>
-  </si>
-  <si>
-    <t xml:space="preserve">N° candidat : </t>
   </si>
   <si>
     <t>Option :</t>
@@ -226,6 +223,15 @@
   </si>
   <si>
     <t>Adresse URL du portfolio : https://samuelcharbit0.github.io/samuelcharbit-portfolio/</t>
+  </si>
+  <si>
+    <t>Création d'un portfolio (HTML, CSS, JS)</t>
+  </si>
+  <si>
+    <t>Sept 2024 - Mars 2025</t>
+  </si>
+  <si>
+    <t>N° candidat : 02541474363</t>
   </si>
 </sst>
 </file>
@@ -311,7 +317,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -706,12 +712,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -806,6 +840,15 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -855,6 +898,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1183,7 +1229,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ82"/>
+  <dimension ref="A1:AQ83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
@@ -1194,124 +1240,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="32"/>
+      <c r="H1" s="35"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="39" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3" s="34"/>
-      <c r="H3" s="40"/>
+      <c r="A3" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="42" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" s="37"/>
+      <c r="H3" s="43"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="36" t="s">
-        <v>35</v>
-      </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="38"/>
+      <c r="A4" s="39" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="H4" s="12" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="56" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="57"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="58"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="12" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="52" t="s">
-        <v>55</v>
-      </c>
-      <c r="B5" s="53"/>
-      <c r="C5" s="53"/>
-      <c r="D5" s="53"/>
-      <c r="E5" s="53"/>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
-      <c r="H5" s="54"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="41" t="s">
+      <c r="B6" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="50" t="s">
+      <c r="C6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="7" t="s">
+    </row>
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="45"/>
+      <c r="B7" s="55"/>
+      <c r="C7" s="13" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="42"/>
-      <c r="B7" s="51"/>
-      <c r="C7" s="13" t="s">
+      <c r="D7" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="E7" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="F7" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="G7" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="H7" s="14" t="s">
         <v>18</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>19</v>
       </c>
       <c r="I7"/>
       <c r="J7"/>
@@ -1350,16 +1396,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="43" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="44"/>
-      <c r="C8" s="45"/>
-      <c r="D8" s="45"/>
-      <c r="E8" s="45"/>
-      <c r="F8" s="45"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="46"/>
+      <c r="A8" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="47"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="48"/>
+      <c r="H8" s="49"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1398,24 +1444,24 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C9" s="26"/>
       <c r="D9" s="25"/>
       <c r="E9" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G9" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H9" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I9"/>
       <c r="J9"/>
@@ -1455,22 +1501,20 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C10" s="26"/>
       <c r="D10" s="25"/>
-      <c r="E10" s="25" t="s">
-        <v>33</v>
-      </c>
+      <c r="E10" s="25"/>
       <c r="F10" s="25"/>
       <c r="G10" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H10" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I10"/>
       <c r="J10"/>
@@ -1510,22 +1554,20 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C11" s="25"/>
       <c r="D11" s="25"/>
-      <c r="E11" s="25" t="s">
-        <v>33</v>
-      </c>
+      <c r="E11" s="25"/>
       <c r="F11" s="25"/>
       <c r="G11" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H11" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I11"/>
       <c r="J11"/>
@@ -1565,22 +1607,20 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C12" s="25"/>
       <c r="D12" s="25"/>
-      <c r="E12" s="25" t="s">
-        <v>33</v>
-      </c>
+      <c r="E12" s="25"/>
       <c r="F12" s="25"/>
       <c r="G12" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H12" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I12"/>
       <c r="J12"/>
@@ -1620,24 +1660,24 @@
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C13" s="25"/>
       <c r="D13" s="25"/>
       <c r="E13" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G13" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H13" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I13"/>
       <c r="J13"/>
@@ -1677,26 +1717,26 @@
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D14" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E14" s="25"/>
       <c r="F14" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G14" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H14" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I14"/>
       <c r="J14"/>
@@ -1736,24 +1776,24 @@
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C15" s="25"/>
       <c r="D15" s="25"/>
       <c r="E15" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F15" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G15" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H15" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I15"/>
       <c r="J15"/>
@@ -1793,22 +1833,22 @@
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C16" s="25"/>
       <c r="D16" s="25"/>
-      <c r="E16" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25" t="s">
+        <v>32</v>
+      </c>
       <c r="G16" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H16" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I16"/>
       <c r="J16"/>
@@ -1848,24 +1888,24 @@
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C17" s="25"/>
       <c r="D17" s="25"/>
       <c r="E17" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F17" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G17" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H17" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I17"/>
       <c r="J17"/>
@@ -1905,28 +1945,28 @@
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E18" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F18" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G18" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H18" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I18"/>
       <c r="J18"/>
@@ -1966,24 +2006,24 @@
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="52.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C19" s="25"/>
       <c r="D19" s="25"/>
       <c r="E19" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F19" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H19" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
+      </c>
+      <c r="H19" s="33" t="s">
+        <v>32</v>
       </c>
       <c r="I19"/>
       <c r="J19"/>
@@ -2021,17 +2061,23 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="47" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="48"/>
-      <c r="C20" s="48"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="48"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="48"/>
-      <c r="H20" s="49"/>
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="G20" s="32"/>
+      <c r="H20" s="34" t="s">
+        <v>32</v>
+      </c>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -2068,27 +2114,17 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="31.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="B21" s="28" t="s">
-        <v>50</v>
-      </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="F21" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="G21" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H21" s="27" t="s">
-        <v>33</v>
-      </c>
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="51"/>
+      <c r="C21" s="51"/>
+      <c r="D21" s="51"/>
+      <c r="E21" s="51"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="51"/>
+      <c r="H21" s="52"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -2125,28 +2161,26 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="31.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="C22" s="25" t="s">
-        <v>33</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" s="10"/>
       <c r="D22" s="10"/>
       <c r="E22" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F22" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G22" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H22" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I22"/>
       <c r="J22"/>
@@ -2186,24 +2220,26 @@
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
+      <c r="E23" s="25" t="s">
+        <v>32</v>
+      </c>
       <c r="F23" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G23" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H23" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I23"/>
       <c r="J23"/>
@@ -2232,18 +2268,36 @@
       <c r="AG23"/>
       <c r="AH23"/>
       <c r="AI23"/>
+      <c r="AJ23"/>
+      <c r="AK23"/>
+      <c r="AL23"/>
+      <c r="AM23"/>
+      <c r="AN23"/>
+      <c r="AO23"/>
+      <c r="AP23"/>
+      <c r="AQ23"/>
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="47" t="s">
-        <v>22</v>
-      </c>
-      <c r="B24" s="48"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="48"/>
-      <c r="H24" s="49"/>
+      <c r="A24" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="G24" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="H24" s="27" t="s">
+        <v>32</v>
+      </c>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -2273,26 +2327,16 @@
       <c r="AI24"/>
     </row>
     <row r="25" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="B25" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="F25" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="G25" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H25" s="27" t="s">
-        <v>33</v>
-      </c>
+      <c r="A25" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="51"/>
+      <c r="C25" s="51"/>
+      <c r="D25" s="51"/>
+      <c r="E25" s="51"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="51"/>
+      <c r="H25" s="53"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2320,37 +2364,27 @@
       <c r="AG25"/>
       <c r="AH25"/>
       <c r="AI25"/>
-      <c r="AJ25"/>
-      <c r="AK25"/>
-      <c r="AL25"/>
-      <c r="AM25"/>
-      <c r="AN25"/>
-      <c r="AO25"/>
-      <c r="AP25"/>
-      <c r="AQ25"/>
-    </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="21" t="s">
-        <v>38</v>
+    </row>
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="15" t="s">
+        <v>36</v>
       </c>
       <c r="B26" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="25" t="s">
-        <v>33</v>
-      </c>
+      <c r="C26" s="10"/>
       <c r="D26" s="10"/>
       <c r="E26" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F26" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G26" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H26" s="27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I26"/>
       <c r="J26"/>
@@ -2388,25 +2422,29 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="49.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="B27" s="30" t="s">
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="29" t="s">
         <v>51</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="D27" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E27" s="25"/>
-      <c r="F27" s="10"/>
+        <v>32</v>
+      </c>
+      <c r="D27" s="10"/>
+      <c r="E27" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="F27" s="25" t="s">
+        <v>32</v>
+      </c>
       <c r="G27" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H27" s="11"/>
+        <v>32</v>
+      </c>
+      <c r="H27" s="27" t="s">
+        <v>32</v>
+      </c>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2443,15 +2481,25 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="5"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="49.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="31" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="D28" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="E28" s="25"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="H28" s="11"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2489,14 +2537,14 @@
       <c r="AQ28"/>
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29"/>
-      <c r="B29"/>
-      <c r="C29"/>
-      <c r="D29"/>
-      <c r="E29"/>
-      <c r="F29"/>
-      <c r="G29"/>
-      <c r="H29"/>
+      <c r="A29" s="5"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2803,7 +2851,7 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36"/>
       <c r="B36"/>
       <c r="C36"/>
@@ -2848,7 +2896,51 @@
       <c r="AP36"/>
       <c r="AQ36"/>
     </row>
-    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="1:43" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37"/>
+      <c r="B37"/>
+      <c r="C37"/>
+      <c r="D37"/>
+      <c r="E37"/>
+      <c r="F37"/>
+      <c r="G37"/>
+      <c r="H37"/>
+      <c r="I37"/>
+      <c r="J37"/>
+      <c r="K37"/>
+      <c r="L37"/>
+      <c r="M37"/>
+      <c r="N37"/>
+      <c r="O37"/>
+      <c r="P37"/>
+      <c r="Q37"/>
+      <c r="R37"/>
+      <c r="S37"/>
+      <c r="T37"/>
+      <c r="U37"/>
+      <c r="V37"/>
+      <c r="W37"/>
+      <c r="X37"/>
+      <c r="Y37"/>
+      <c r="Z37"/>
+      <c r="AA37"/>
+      <c r="AB37"/>
+      <c r="AC37"/>
+      <c r="AD37"/>
+      <c r="AE37"/>
+      <c r="AF37"/>
+      <c r="AG37"/>
+      <c r="AH37"/>
+      <c r="AI37"/>
+      <c r="AJ37"/>
+      <c r="AK37"/>
+      <c r="AL37"/>
+      <c r="AM37"/>
+      <c r="AN37"/>
+      <c r="AO37"/>
+      <c r="AP37"/>
+      <c r="AQ37"/>
+    </row>
     <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -2886,16 +2978,7 @@
     <row r="72" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="73" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="74" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="1"/>
-      <c r="B75" s="1"/>
-      <c r="C75" s="1"/>
-      <c r="D75" s="1"/>
-      <c r="E75" s="1"/>
-      <c r="F75" s="1"/>
-      <c r="G75" s="1"/>
-      <c r="H75" s="1"/>
-    </row>
+    <row r="75" spans="1:8" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="76" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
@@ -2966,13 +3049,23 @@
       <c r="G82" s="1"/>
       <c r="H82" s="1"/>
     </row>
+    <row r="83" spans="1:8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="1"/>
+      <c r="B83" s="1"/>
+      <c r="C83" s="1"/>
+      <c r="D83" s="1"/>
+      <c r="E83" s="1"/>
+      <c r="F83" s="1"/>
+      <c r="G83" s="1"/>
+      <c r="H83" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A25:H25"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="G1:H1"/>

</xml_diff>

<commit_message>
Modif tableau de synthèse
</commit_message>
<xml_diff>
--- a/public/Tableau de synthese.xlsx
+++ b/public/Tableau de synthese.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1E34428-B898-4FA9-987F-F34C0426BCBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F599CA5-54C5-433B-BF1E-C4AA6D532595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -228,10 +228,10 @@
     <t>Création d'un portfolio (HTML, CSS, JS)</t>
   </si>
   <si>
-    <t>Sept 2024 - Mars 2025</t>
-  </si>
-  <si>
     <t>N° candidat : 02541474363</t>
+  </si>
+  <si>
+    <t>Sept 2024 - Mars 2026</t>
   </si>
 </sst>
 </file>
@@ -849,9 +849,54 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -874,51 +919,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1240,56 +1240,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="35"/>
+      <c r="H1" s="37"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="42" t="s">
-        <v>57</v>
-      </c>
-      <c r="G3" s="37"/>
-      <c r="H3" s="43"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="52"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="57" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="52"/>
+      <c r="H3" s="58"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="54" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="41"/>
+      <c r="B4" s="55"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="56"/>
       <c r="F4" s="8" t="s">
         <v>3</v>
       </c>
@@ -1301,22 +1301,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="56" t="s">
+      <c r="A5" s="48" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="57"/>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="58"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="50"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="44" t="s">
+      <c r="A6" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="46" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1339,8 +1339,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="45"/>
-      <c r="B7" s="55"/>
+      <c r="A7" s="36"/>
+      <c r="B7" s="47"/>
       <c r="C7" s="13" t="s">
         <v>13</v>
       </c>
@@ -1396,16 +1396,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="46" t="s">
+      <c r="A8" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="47"/>
-      <c r="C8" s="48"/>
-      <c r="D8" s="48"/>
-      <c r="E8" s="48"/>
-      <c r="F8" s="48"/>
-      <c r="G8" s="48"/>
-      <c r="H8" s="49"/>
+      <c r="B8" s="39"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="41"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -2066,7 +2066,7 @@
         <v>55</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
@@ -2115,16 +2115,16 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="50" t="s">
+      <c r="A21" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="51"/>
-      <c r="C21" s="51"/>
-      <c r="D21" s="51"/>
-      <c r="E21" s="51"/>
-      <c r="F21" s="51"/>
-      <c r="G21" s="51"/>
-      <c r="H21" s="52"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="44"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -2327,16 +2327,16 @@
       <c r="AI24"/>
     </row>
     <row r="25" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="50" t="s">
+      <c r="A25" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="51"/>
-      <c r="C25" s="51"/>
-      <c r="D25" s="51"/>
-      <c r="E25" s="51"/>
-      <c r="F25" s="51"/>
-      <c r="G25" s="51"/>
-      <c r="H25" s="53"/>
+      <c r="B25" s="43"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="43"/>
+      <c r="F25" s="43"/>
+      <c r="G25" s="43"/>
+      <c r="H25" s="45"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -3061,6 +3061,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -3068,11 +3073,6 @@
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -3278,6 +3278,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="b51e6d1e-8224-46a7-86ba-7d6901891049" xsi:nil="true"/>
@@ -3286,15 +3295,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3317,6 +3317,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E5CC2F8-6A3D-4E00-BE87-ABD27B2DABA8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{092602E4-9251-40C3-8AA3-A273484EC6BA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3325,12 +3333,4 @@
     <ds:schemaRef ds:uri="8955dbd3-594d-423f-94ea-9d3376d0dae5"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E5CC2F8-6A3D-4E00-BE87-ABD27B2DABA8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>